<commit_message>
SupplyScope: fix reviewer findings R3-01..R3-07 and S-02/S-03 (SKU-day stockout metric with calendar-day share, scenario-scoped unmet demand with 409 conflicts, dataset-version staleness and stale drafts, multi-location position, microsecond instants, target >= ROP, negative-available flag and BIGINT sums, supplier load order, promo factor 1+uplift); D-07 and amendments; regression tests in Python, SQL and TypeScript; artifacts regenerated
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018qazUm6EuWcx7grXhz8gRg
</commit_message>
<xml_diff>
--- a/apps/supplyscope/artifacts/supplyscope-analyst-workbook.xlsx
+++ b/apps/supplyscope/artifacts/supplyscope-analyst-workbook.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="953" uniqueCount="391">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="955" uniqueCount="393">
   <si>
     <t xml:space="preserve">Inputs: the golden fixture (tests/fixtures/golden/inputs.json, fixture supplyscope-golden-v1)</t>
   </si>
@@ -1126,13 +1126,13 @@
     <t xml:space="preserve">Stockout SKU Day Share</t>
   </si>
   <si>
-    <t xml:space="preserve">431 / 32880, query 03 ALL</t>
+    <t xml:space="preserve">431 / 32880, query 03 ALL, reference_metrics.sql stockout_days</t>
   </si>
   <si>
     <t xml:space="preserve">Stockout Calendar Day Share</t>
   </si>
   <si>
-    <t xml:space="preserve">290 / 548, reference_metrics.sql stockout_days</t>
+    <t xml:space="preserve">290 / 548, reference_metrics.sql stockout_calendar_days_share</t>
   </si>
   <si>
     <t xml:space="preserve">On Hand Units (2026-09-30)</t>
@@ -1190,6 +1190,12 @@
   </si>
   <si>
     <t xml:space="preserve">available</t>
+  </si>
+  <si>
+    <t xml:space="preserve">stockout_calendar_days_share</t>
+  </si>
+  <si>
+    <t xml:space="preserve">observed_sku_days</t>
   </si>
   <si>
     <t xml:space="preserve">reconciliation (run_all.py): checks equal / checks run</t>
@@ -3677,7 +3683,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:X314"/>
+  <dimension ref="A1:Z314"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="26"/>
@@ -11032,7 +11038,7 @@
       <c r="Q307" s="14"/>
       <c r="R307" s="14"/>
     </row>
-    <row r="308" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="308" customFormat="false" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A308" s="3" t="s">
         <v>227</v>
       </c>
@@ -11104,6 +11110,12 @@
       </c>
       <c r="X308" s="3" t="s">
         <v>314</v>
+      </c>
+      <c r="Y308" s="3" t="s">
+        <v>388</v>
+      </c>
+      <c r="Z308" s="3" t="s">
+        <v>389</v>
       </c>
     </row>
     <row r="309" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11123,10 +11135,10 @@
         <v>548</v>
       </c>
       <c r="F309" s="0" t="n">
-        <v>290</v>
+        <v>431</v>
       </c>
       <c r="G309" s="0" t="n">
-        <v>0.529197</v>
+        <v>0.013108</v>
       </c>
       <c r="H309" s="0" t="n">
         <v>0</v>
@@ -11179,10 +11191,16 @@
       <c r="X309" s="0" t="n">
         <v>240</v>
       </c>
+      <c r="Y309" s="0" t="n">
+        <v>0.529197</v>
+      </c>
+      <c r="Z309" s="0" t="n">
+        <v>32880</v>
+      </c>
     </row>
     <row r="312" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A312" s="13" t="s">
-        <v>388</v>
+        <v>390</v>
       </c>
       <c r="B312" s="14"/>
       <c r="C312" s="14"/>
@@ -11204,18 +11222,18 @@
     </row>
     <row r="313" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A313" s="3" t="s">
-        <v>389</v>
+        <v>391</v>
       </c>
       <c r="B313" s="3" t="s">
-        <v>390</v>
+        <v>392</v>
       </c>
     </row>
     <row r="314" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A314" s="0" t="n">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="B314" s="0" t="n">
-        <v>87</v>
+        <v>91</v>
       </c>
     </row>
   </sheetData>

</xml_diff>